<commit_message>
Link settlement accounts to assigned idols
</commit_message>
<xml_diff>
--- a/sample-data/사원정보/Food-Fee_더미_사원_로그인_계정.xlsx
+++ b/sample-data/사원정보/Food-Fee_더미_사원_로그인_계정.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="로그인 계정" sheetId="1" r:id="R11ee90ef0e264855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="로그인 계정" sheetId="1" r:id="R391809f17d8a445b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +16,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="@"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -55,8 +55,28 @@
       <x:color rgb="FF155866"/>
       <x:name val="맑은 고딕"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF263238"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1B7F5A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF64717D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF28718A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -83,8 +103,28 @@
         <x:fgColor rgb="FFE9EEF1"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="10">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -159,11 +199,25 @@
         <x:color rgb="FFDFE6EA"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2E8"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2E8"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2E8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2E8"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="61">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -269,6 +323,39 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -312,8 +399,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LoginAccountsTable" displayName="LoginAccountsTable" ref="A5:I8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:I8"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LoginAccountsTable" displayName="LoginAccountsTable" ref="A5:I9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:I9"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="사번"/>
     <x:tableColumn id="2" name="성명"/>
@@ -563,7 +650,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="17" t="str">
-        <x:v>작성 기준일: 2026-07-15 · 비밀번호 규칙: 사번 마지막 4자리 · 앱 로그인 계정과 동일</x:v>
+        <x:v>작성 기준일: 2026-07-15, 비밀번호 규칙: 사번 마지막 4자리, 앱 로그인 계정과 동일</x:v>
       </x:c>
       <x:c r="B3" s="17"/>
       <x:c r="C3" s="17"/>
@@ -608,7 +695,7 @@
         <x:v>FIN-1024</x:v>
       </x:c>
       <x:c r="B6" s="37" t="str">
-        <x:v>정산 담당자</x:v>
+        <x:v>삼일돌 정산 담당자</x:v>
       </x:c>
       <x:c r="C6" s="37" t="str">
         <x:v>정산 담당자</x:v>
@@ -630,7 +717,7 @@
         <x:v>활성</x:v>
       </x:c>
       <x:c r="I6" s="39" t="str">
-        <x:v>현재 아이돌 식비 정산 전용 · 지급 정산금액/로그 비공개</x:v>
+        <x:v>삼일돌(Samildol) 식비 정산 전용, 지급 정산금액/로그 비공개</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -660,7 +747,7 @@
         <x:v>활성</x:v>
       </x:c>
       <x:c r="I7" s="40" t="str">
-        <x:v>정산 입력·Excel 출력 가능 · 승인/로그 열람 불가</x:v>
+        <x:v>정산 입력, Excel 출력 가능, 승인/로그 열람 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
@@ -690,7 +777,36 @@
         <x:v>활성</x:v>
       </x:c>
       <x:c r="I8" s="40" t="str">
-        <x:v>모든 권한 보유 · 승인 버튼 및 감사 로그 열람 가능</x:v>
+        <x:v>모든 권한 보유, 승인 버튼 및 감사 로그 열람 가능</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="27" customHeight="1">
+      <x:c r="A9" s="52" t="str">
+        <x:v>FIN-1025</x:v>
+      </x:c>
+      <x:c r="B9" s="52" t="str">
+        <x:v>삼데헌 정산 담당자</x:v>
+      </x:c>
+      <x:c r="C9" s="52" t="str">
+        <x:v>정산 담당자</x:v>
+      </x:c>
+      <x:c r="D9" s="52" t="str">
+        <x:v>1025</x:v>
+      </x:c>
+      <x:c r="E9" s="54" t="str">
+        <x:v>있음</x:v>
+      </x:c>
+      <x:c r="F9" s="56" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="G9" s="56" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="H9" s="58" t="str">
+        <x:v>활성</x:v>
+      </x:c>
+      <x:c r="I9" s="60" t="str">
+        <x:v>삼데헌 식비 정산 전용, 지급 정산금액/로그 비공개</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26" customHeight="1">
@@ -721,7 +837,7 @@
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="47" t="str">
-        <x:v>2. 로그인·로그아웃·권한 차단 이력은 Food-Fee 감사 로그에 기록됩니다.</x:v>
+        <x:v>2. 로그인, 로그아웃, 권한 차단 이력은 Food-Fee 감사 로그에 기록됩니다.</x:v>
       </x:c>
       <x:c r="B12" s="47"/>
       <x:c r="C12" s="47"/>
@@ -749,11 +865,11 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>
     <x:mergeCell ref="A2:I2"/>
-    <x:mergeCell ref="A3:I3"/>
     <x:mergeCell ref="A10:I10"/>
     <x:mergeCell ref="A11:I11"/>
     <x:mergeCell ref="A12:I12"/>
     <x:mergeCell ref="A13:I13"/>
+    <x:mergeCell ref="A3:I3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="E6:G8">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="있음"/>
@@ -769,7 +885,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5035155cbf79473b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ddb7aa3723e4f97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Rename field managers and restrict payroll visibility
</commit_message>
<xml_diff>
--- a/sample-data/사원정보/Food-Fee_더미_사원_로그인_계정.xlsx
+++ b/sample-data/사원정보/Food-Fee_더미_사원_로그인_계정.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="로그인 계정" sheetId="1" r:id="R391809f17d8a445b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="로그인 계정" sheetId="1" r:id="Rdef3d97bdd29444b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -695,10 +695,10 @@
         <x:v>FIN-1024</x:v>
       </x:c>
       <x:c r="B6" s="37" t="str">
-        <x:v>삼일돌 정산 담당자</x:v>
+        <x:v>삼일돌 현장 매니저</x:v>
       </x:c>
       <x:c r="C6" s="37" t="str">
-        <x:v>정산 담당자</x:v>
+        <x:v>현장 매니저</x:v>
       </x:c>
       <x:c r="D6" s="41" t="str">
         <x:f>RIGHT(A6,4)</x:f>
@@ -785,10 +785,10 @@
         <x:v>FIN-1025</x:v>
       </x:c>
       <x:c r="B9" s="52" t="str">
-        <x:v>삼데헌 정산 담당자</x:v>
+        <x:v>삼데헌 현장 매니저</x:v>
       </x:c>
       <x:c r="C9" s="52" t="str">
-        <x:v>정산 담당자</x:v>
+        <x:v>현장 매니저</x:v>
       </x:c>
       <x:c r="D9" s="52" t="str">
         <x:v>1025</x:v>
@@ -885,7 +885,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ddb7aa3723e4f97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R389cb311b6d0436d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Replace xlsx export with idol import
</commit_message>
<xml_diff>
--- a/sample-data/사원정보/Food-Fee_더미_사원_로그인_계정.xlsx
+++ b/sample-data/사원정보/Food-Fee_더미_사원_로그인_계정.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="로그인 계정" sheetId="1" r:id="Rdef3d97bdd29444b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="로그인 계정" sheetId="1" r:id="Rf16d945803dd43e4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +16,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="@"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="21">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -75,8 +75,63 @@
       <x:color rgb="FF28718A"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF27343A"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF27343A"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="20"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF805B00"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF687983"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF18856B"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF687983"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF277391"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF155E6B"/>
+      <x:name val="Malgun Gothic"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="28">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +176,96 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF155E6B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2C9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF238196"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC9EAF6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F4F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7EEF1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF155E6B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2C9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF238196"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC9EAF6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F4F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAF5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7EEF1"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -217,7 +362,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="61">
+  <x:cellXfs count="219">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -356,6 +501,476 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="15" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="15" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="15" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="15" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="16" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="16" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="16" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="16" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="16" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="16" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="17" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="17" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="17" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="17" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="19" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="19" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="19" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="19" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="19" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="19" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="19" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="19" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="19" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="21" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="21" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="22" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="22" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="22" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="23" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="23" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="23" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="12" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="24" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="24" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="24" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="24" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="24" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="24" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="25" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="25" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="25" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="25" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="25" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="25" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="26" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="26" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="26" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="26" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -622,244 +1237,255 @@
     <x:col min="9" max="9" width="35" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+    <x:row r="1" ht="33" customHeight="1">
+      <x:c r="A1" s="180" t="str">
         <x:v>Food-Fee 더미 사원 로그인 계정</x:v>
       </x:c>
-      <x:c r="B1" s="4"/>
-      <x:c r="C1" s="4"/>
-      <x:c r="D1" s="4"/>
-      <x:c r="E1" s="4"/>
-      <x:c r="F1" s="4"/>
-      <x:c r="G1" s="4"/>
-      <x:c r="H1" s="4"/>
-      <x:c r="I1" s="4"/>
+      <x:c r="B1" s="180"/>
+      <x:c r="C1" s="180"/>
+      <x:c r="D1" s="180"/>
+      <x:c r="E1" s="180"/>
+      <x:c r="F1" s="180"/>
+      <x:c r="G1" s="180"/>
+      <x:c r="H1" s="180"/>
+      <x:c r="I1" s="180"/>
     </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="13" t="str">
+    <x:row r="2" ht="25.5" customHeight="1">
+      <x:c r="A2" s="184" t="str">
         <x:v>보안 안내: 아래 비밀번호는 PoC 테스트용 평문 더미 데이터입니다. 실제 사내 계정이나 운영 환경에서 사용하지 마세요.</x:v>
       </x:c>
-      <x:c r="B2" s="14"/>
-      <x:c r="C2" s="14"/>
-      <x:c r="D2" s="14"/>
-      <x:c r="E2" s="14"/>
-      <x:c r="F2" s="14"/>
-      <x:c r="G2" s="14"/>
-      <x:c r="H2" s="14"/>
-      <x:c r="I2" s="15"/>
+      <x:c r="B2" s="185"/>
+      <x:c r="C2" s="185"/>
+      <x:c r="D2" s="185"/>
+      <x:c r="E2" s="185"/>
+      <x:c r="F2" s="185"/>
+      <x:c r="G2" s="185"/>
+      <x:c r="H2" s="185"/>
+      <x:c r="I2" s="186"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="17" t="str">
+      <x:c r="A3" s="147" t="str">
         <x:v>작성 기준일: 2026-07-15, 비밀번호 규칙: 사번 마지막 4자리, 앱 로그인 계정과 동일</x:v>
       </x:c>
-      <x:c r="B3" s="17"/>
-      <x:c r="C3" s="17"/>
-      <x:c r="D3" s="17"/>
-      <x:c r="E3" s="17"/>
-      <x:c r="F3" s="17"/>
-      <x:c r="G3" s="17"/>
-      <x:c r="H3" s="17"/>
-      <x:c r="I3" s="17"/>
+      <x:c r="B3" s="147"/>
+      <x:c r="C3" s="147"/>
+      <x:c r="D3" s="147"/>
+      <x:c r="E3" s="147"/>
+      <x:c r="F3" s="147"/>
+      <x:c r="G3" s="147"/>
+      <x:c r="H3" s="147"/>
+      <x:c r="I3" s="147"/>
     </x:row>
-    <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="29" t="str">
+    <x:row r="4">
+      <x:c r="A4" s="148"/>
+      <x:c r="B4" s="148"/>
+      <x:c r="C4" s="148"/>
+      <x:c r="D4" s="148"/>
+      <x:c r="E4" s="148"/>
+      <x:c r="F4" s="148"/>
+      <x:c r="G4" s="148"/>
+      <x:c r="H4" s="148"/>
+      <x:c r="I4" s="148"/>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="190" t="str">
         <x:v>사번</x:v>
       </x:c>
-      <x:c r="B5" s="30" t="str">
+      <x:c r="B5" s="191" t="str">
         <x:v>성명</x:v>
       </x:c>
-      <x:c r="C5" s="30" t="str">
+      <x:c r="C5" s="191" t="str">
         <x:v>역할</x:v>
       </x:c>
-      <x:c r="D5" s="30" t="str">
+      <x:c r="D5" s="191" t="str">
         <x:v>더미 비밀번호</x:v>
       </x:c>
-      <x:c r="E5" s="30" t="str">
+      <x:c r="E5" s="191" t="str">
         <x:v>입력 권한</x:v>
       </x:c>
-      <x:c r="F5" s="30" t="str">
-        <x:v>Excel 출력 권한</x:v>
-      </x:c>
-      <x:c r="G5" s="30" t="str">
+      <x:c r="F5" s="191" t="str">
+        <x:v>다른 아이돌 연동</x:v>
+      </x:c>
+      <x:c r="G5" s="191" t="str">
         <x:v>승인 권한</x:v>
       </x:c>
-      <x:c r="H5" s="30" t="str">
+      <x:c r="H5" s="191" t="str">
         <x:v>계정 상태</x:v>
       </x:c>
-      <x:c r="I5" s="31" t="str">
+      <x:c r="I5" s="192" t="str">
         <x:v>비고</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="28" customHeight="1">
-      <x:c r="A6" s="37" t="str">
+    <x:row r="6" ht="31.5" customHeight="1">
+      <x:c r="A6" s="193" t="str">
         <x:v>FIN-1024</x:v>
       </x:c>
-      <x:c r="B6" s="37" t="str">
+      <x:c r="B6" s="193" t="str">
         <x:v>삼일돌 현장 매니저</x:v>
       </x:c>
-      <x:c r="C6" s="37" t="str">
+      <x:c r="C6" s="193" t="str">
         <x:v>현장 매니저</x:v>
       </x:c>
-      <x:c r="D6" s="41" t="str">
+      <x:c r="D6" s="194" t="str">
         <x:f>RIGHT(A6,4)</x:f>
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E6" s="37" t="str">
+      <x:c r="E6" s="202" t="str">
         <x:v>있음</x:v>
       </x:c>
-      <x:c r="F6" s="37" t="str">
+      <x:c r="F6" s="206" t="str">
         <x:v>없음</x:v>
       </x:c>
-      <x:c r="G6" s="37" t="str">
+      <x:c r="G6" s="206" t="str">
         <x:v>없음</x:v>
       </x:c>
-      <x:c r="H6" s="37" t="str">
+      <x:c r="H6" s="214" t="str">
         <x:v>활성</x:v>
       </x:c>
-      <x:c r="I6" s="39" t="str">
+      <x:c r="I6" s="195" t="str">
         <x:v>삼일돌(Samildol) 식비 정산 전용, 지급 정산금액/로그 비공개</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="28" customHeight="1">
-      <x:c r="A7" s="38" t="str">
+    <x:row r="7" ht="31.5" customHeight="1">
+      <x:c r="A7" s="158" t="str">
         <x:v>MGR-2201</x:v>
       </x:c>
-      <x:c r="B7" s="38" t="str">
+      <x:c r="B7" s="158" t="str">
         <x:v>상위 매니저</x:v>
       </x:c>
-      <x:c r="C7" s="38" t="str">
+      <x:c r="C7" s="158" t="str">
         <x:v>상위 매니저</x:v>
       </x:c>
-      <x:c r="D7" s="42" t="str">
+      <x:c r="D7" s="159" t="str">
         <x:f>RIGHT(A7,4)</x:f>
         <x:v>2201</x:v>
       </x:c>
-      <x:c r="E7" s="38" t="str">
+      <x:c r="E7" s="203" t="str">
         <x:v>있음</x:v>
       </x:c>
-      <x:c r="F7" s="38" t="str">
+      <x:c r="F7" s="203" t="str">
         <x:v>있음</x:v>
       </x:c>
-      <x:c r="G7" s="38" t="str">
+      <x:c r="G7" s="208" t="str">
         <x:v>없음</x:v>
       </x:c>
-      <x:c r="H7" s="38" t="str">
+      <x:c r="H7" s="215" t="str">
         <x:v>활성</x:v>
       </x:c>
-      <x:c r="I7" s="40" t="str">
-        <x:v>정산 입력, Excel 출력 가능, 승인/로그 열람 불가</x:v>
+      <x:c r="I7" s="163" t="str">
+        <x:v>정산 입력, 다른 아이돌 .xlsx 연동 가능, 승인/로그 열람 불가</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="38" t="str">
+    <x:row r="8" ht="31.5" customHeight="1">
+      <x:c r="A8" s="196" t="str">
         <x:v>HR-3007</x:v>
       </x:c>
-      <x:c r="B8" s="38" t="str">
+      <x:c r="B8" s="196" t="str">
         <x:v>인사 마스터</x:v>
       </x:c>
-      <x:c r="C8" s="38" t="str">
+      <x:c r="C8" s="196" t="str">
         <x:v>내부 데이터 관리자</x:v>
       </x:c>
-      <x:c r="D8" s="42" t="str">
+      <x:c r="D8" s="197" t="str">
         <x:f>RIGHT(A8,4)</x:f>
         <x:v>3007</x:v>
       </x:c>
-      <x:c r="E8" s="38" t="str">
+      <x:c r="E8" s="203" t="str">
         <x:v>있음</x:v>
       </x:c>
-      <x:c r="F8" s="38" t="str">
+      <x:c r="F8" s="203" t="str">
         <x:v>있음</x:v>
       </x:c>
-      <x:c r="G8" s="38" t="str">
+      <x:c r="G8" s="203" t="str">
         <x:v>있음</x:v>
       </x:c>
-      <x:c r="H8" s="38" t="str">
+      <x:c r="H8" s="215" t="str">
         <x:v>활성</x:v>
       </x:c>
-      <x:c r="I8" s="40" t="str">
-        <x:v>모든 권한 보유, 승인 버튼 및 감사 로그 열람 가능</x:v>
+      <x:c r="I8" s="198" t="str">
+        <x:v>전체 데이터 입력, 다른 아이돌 .xlsx 연동, 승인 및 감사 로그 열람 가능</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="27" customHeight="1">
-      <x:c r="A9" s="52" t="str">
+    <x:row r="9" ht="31.5" customHeight="1">
+      <x:c r="A9" s="164" t="str">
         <x:v>FIN-1025</x:v>
       </x:c>
-      <x:c r="B9" s="52" t="str">
+      <x:c r="B9" s="164" t="str">
         <x:v>삼데헌 현장 매니저</x:v>
       </x:c>
-      <x:c r="C9" s="52" t="str">
+      <x:c r="C9" s="164" t="str">
         <x:v>현장 매니저</x:v>
       </x:c>
-      <x:c r="D9" s="52" t="str">
+      <x:c r="D9" s="164" t="str">
         <x:v>1025</x:v>
       </x:c>
-      <x:c r="E9" s="54" t="str">
+      <x:c r="E9" s="204" t="str">
         <x:v>있음</x:v>
       </x:c>
-      <x:c r="F9" s="56" t="str">
+      <x:c r="F9" s="210" t="str">
         <x:v>없음</x:v>
       </x:c>
-      <x:c r="G9" s="56" t="str">
+      <x:c r="G9" s="210" t="str">
         <x:v>없음</x:v>
       </x:c>
-      <x:c r="H9" s="58" t="str">
+      <x:c r="H9" s="216" t="str">
         <x:v>활성</x:v>
       </x:c>
-      <x:c r="I9" s="60" t="str">
+      <x:c r="I9" s="168" t="str">
         <x:v>삼데헌 식비 정산 전용, 지급 정산금액/로그 비공개</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="26" customHeight="1">
-      <x:c r="A10" s="45" t="str">
+      <x:c r="A10" s="218" t="str">
         <x:v>계정 운영 메모</x:v>
       </x:c>
-      <x:c r="B10" s="45"/>
-      <x:c r="C10" s="45"/>
-      <x:c r="D10" s="45"/>
-      <x:c r="E10" s="45"/>
-      <x:c r="F10" s="45"/>
-      <x:c r="G10" s="45"/>
-      <x:c r="H10" s="45"/>
-      <x:c r="I10" s="45"/>
+      <x:c r="B10" s="218"/>
+      <x:c r="C10" s="218"/>
+      <x:c r="D10" s="218"/>
+      <x:c r="E10" s="218"/>
+      <x:c r="F10" s="218"/>
+      <x:c r="G10" s="218"/>
+      <x:c r="H10" s="218"/>
+      <x:c r="I10" s="218"/>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
-      <x:c r="A11" s="47" t="str">
+      <x:c r="A11" s="170" t="str">
         <x:v>1. 로그인 세션은 브라우저 탭을 닫거나 로그아웃할 때 종료됩니다.</x:v>
       </x:c>
-      <x:c r="B11" s="47"/>
-      <x:c r="C11" s="47"/>
-      <x:c r="D11" s="47"/>
-      <x:c r="E11" s="47"/>
-      <x:c r="F11" s="47"/>
-      <x:c r="G11" s="47"/>
-      <x:c r="H11" s="47"/>
-      <x:c r="I11" s="47"/>
+      <x:c r="B11" s="170"/>
+      <x:c r="C11" s="170"/>
+      <x:c r="D11" s="170"/>
+      <x:c r="E11" s="170"/>
+      <x:c r="F11" s="170"/>
+      <x:c r="G11" s="170"/>
+      <x:c r="H11" s="170"/>
+      <x:c r="I11" s="170"/>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
-      <x:c r="A12" s="47" t="str">
+      <x:c r="A12" s="170" t="str">
         <x:v>2. 로그인, 로그아웃, 권한 차단 이력은 Food-Fee 감사 로그에 기록됩니다.</x:v>
       </x:c>
-      <x:c r="B12" s="47"/>
-      <x:c r="C12" s="47"/>
-      <x:c r="D12" s="47"/>
-      <x:c r="E12" s="47"/>
-      <x:c r="F12" s="47"/>
-      <x:c r="G12" s="47"/>
-      <x:c r="H12" s="47"/>
-      <x:c r="I12" s="47"/>
+      <x:c r="B12" s="170"/>
+      <x:c r="C12" s="170"/>
+      <x:c r="D12" s="170"/>
+      <x:c r="E12" s="170"/>
+      <x:c r="F12" s="170"/>
+      <x:c r="G12" s="170"/>
+      <x:c r="H12" s="170"/>
+      <x:c r="I12" s="170"/>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
-      <x:c r="A13" s="47" t="str">
+      <x:c r="A13" s="170" t="str">
         <x:v>3. 실제 배포 시 회사 SSO와 서버 측 세션으로 교체하고 평문 비밀번호 파일은 폐기해야 합니다.</x:v>
       </x:c>
-      <x:c r="B13" s="47"/>
-      <x:c r="C13" s="47"/>
-      <x:c r="D13" s="47"/>
-      <x:c r="E13" s="47"/>
-      <x:c r="F13" s="47"/>
-      <x:c r="G13" s="47"/>
-      <x:c r="H13" s="47"/>
-      <x:c r="I13" s="47"/>
+      <x:c r="B13" s="170"/>
+      <x:c r="C13" s="170"/>
+      <x:c r="D13" s="170"/>
+      <x:c r="E13" s="170"/>
+      <x:c r="F13" s="170"/>
+      <x:c r="G13" s="170"/>
+      <x:c r="H13" s="170"/>
+      <x:c r="I13" s="170"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -885,7 +1511,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R389cb311b6d0436d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9111682b50944cc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>